<commit_message>
correción en la matriz y diagramas
</commit_message>
<xml_diff>
--- a/Documentación/Matriz de CUS.xlsx
+++ b/Documentación/Matriz de CUS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joaquin\Desktop\MelodicVault\Documentación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B45BB217-2E02-4F22-955F-FE5AA539C357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCDD124F-A8A1-4500-95F9-6E2EC5E1ED29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{67580095-C0D5-4242-B9B2-4C035CE11869}"/>
   </bookViews>
@@ -789,7 +789,7 @@
         <v>12</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>16</v>
@@ -823,7 +823,7 @@
         <v>9</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>6</v>

</xml_diff>

<commit_message>
correción de matriz de Cu
</commit_message>
<xml_diff>
--- a/Documentación/Matriz de CUS.xlsx
+++ b/Documentación/Matriz de CUS.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joaquin\Desktop\MelodicVault\Documentación\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joaquin\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCDD124F-A8A1-4500-95F9-6E2EC5E1ED29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{637F6008-5453-4BBB-8DC9-5159AFA0F3D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{67580095-C0D5-4242-B9B2-4C035CE11869}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="70">
   <si>
     <t>Código</t>
   </si>
@@ -137,9 +137,6 @@
     <t>Registrar Canción</t>
   </si>
   <si>
-    <t>Consultar Canción</t>
-  </si>
-  <si>
     <t>CU14</t>
   </si>
   <si>
@@ -152,9 +149,6 @@
     <t>CU17</t>
   </si>
   <si>
-    <t>CU18</t>
-  </si>
-  <si>
     <t>Editar Canción</t>
   </si>
   <si>
@@ -173,9 +167,6 @@
     <t>Registra una canción en el sistema.</t>
   </si>
   <si>
-    <t>Consulta información de una canción registrada en el sistema.</t>
-  </si>
-  <si>
     <t>Modifica la información de una canción registrada en el sistema.</t>
   </si>
   <si>
@@ -209,12 +200,6 @@
     <t>Matriz de Casos de Uso  - MelodicVault</t>
   </si>
   <si>
-    <t>Extiende: CU15, CU18</t>
-  </si>
-  <si>
-    <t>Incluye CU13</t>
-  </si>
-  <si>
     <t>Extiende: CU13</t>
   </si>
   <si>
@@ -261,6 +246,9 @@
   </si>
   <si>
     <t>Consulta información sobre un Álbum registrado en el sistema.</t>
+  </si>
+  <si>
+    <t>Extiende: CU15</t>
   </si>
 </sst>
 </file>
@@ -330,7 +318,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -366,11 +354,33 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -404,6 +414,18 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -756,7 +778,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -795,7 +817,7 @@
         <v>16</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -812,7 +834,7 @@
         <v>15</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -846,7 +868,7 @@
         <v>6</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -854,7 +876,7 @@
         <v>17</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>13</v>
@@ -863,7 +885,7 @@
         <v>6</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -877,10 +899,10 @@
         <v>30</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -894,10 +916,10 @@
         <v>30</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -911,10 +933,10 @@
         <v>13</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -922,7 +944,7 @@
         <v>21</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>30</v>
@@ -931,7 +953,7 @@
         <v>6</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -939,16 +961,16 @@
         <v>22</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -956,16 +978,16 @@
         <v>23</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>30</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -973,16 +995,16 @@
         <v>24</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>30</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -990,21 +1012,21 @@
         <v>25</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>31</v>
@@ -1016,76 +1038,66 @@
         <v>6</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>13</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>30</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C19" s="7" t="s">
+      <c r="A19" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="D19" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>46</v>
+      <c r="D19" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="E20" s="8" t="s">
-        <v>44</v>
-      </c>
+      <c r="A20" s="14"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>